<commit_message>
Add a dedicated PivotTable filter field to test data
</commit_message>
<xml_diff>
--- a/inputs/test_input_100rows.xlsx
+++ b/inputs/test_input_100rows.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Score</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -477,6 +482,11 @@
       <c r="E2" t="n">
         <v>60</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -500,6 +510,11 @@
       <c r="E3" t="n">
         <v>61.5</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,6 +538,11 @@
       <c r="E4" t="n">
         <v>63</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,6 +566,11 @@
       <c r="E5" t="n">
         <v>64.5</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -569,6 +594,11 @@
       <c r="E6" t="n">
         <v>66</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -592,6 +622,11 @@
       <c r="E7" t="n">
         <v>67.5</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -615,6 +650,11 @@
       <c r="E8" t="n">
         <v>69</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -638,6 +678,11 @@
       <c r="E9" t="n">
         <v>70.5</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -661,6 +706,11 @@
       <c r="E10" t="n">
         <v>72</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -684,6 +734,11 @@
       <c r="E11" t="n">
         <v>73.5</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -707,6 +762,11 @@
       <c r="E12" t="n">
         <v>75</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -730,6 +790,11 @@
       <c r="E13" t="n">
         <v>76.5</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -753,6 +818,11 @@
       <c r="E14" t="n">
         <v>78</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -776,6 +846,11 @@
       <c r="E15" t="n">
         <v>79.5</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -799,6 +874,11 @@
       <c r="E16" t="n">
         <v>81</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -822,6 +902,11 @@
       <c r="E17" t="n">
         <v>82.5</v>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -845,6 +930,11 @@
       <c r="E18" t="n">
         <v>84</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -868,6 +958,11 @@
       <c r="E19" t="n">
         <v>60</v>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -891,6 +986,11 @@
       <c r="E20" t="n">
         <v>61.5</v>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -914,6 +1014,11 @@
       <c r="E21" t="n">
         <v>63</v>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -937,6 +1042,11 @@
       <c r="E22" t="n">
         <v>64.5</v>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -960,6 +1070,11 @@
       <c r="E23" t="n">
         <v>66</v>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -983,6 +1098,11 @@
       <c r="E24" t="n">
         <v>67.5</v>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1006,6 +1126,11 @@
       <c r="E25" t="n">
         <v>69</v>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1029,6 +1154,11 @@
       <c r="E26" t="n">
         <v>70.5</v>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1052,6 +1182,11 @@
       <c r="E27" t="n">
         <v>72</v>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1075,6 +1210,11 @@
       <c r="E28" t="n">
         <v>73.5</v>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1098,6 +1238,11 @@
       <c r="E29" t="n">
         <v>75</v>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1121,6 +1266,11 @@
       <c r="E30" t="n">
         <v>76.5</v>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1144,6 +1294,11 @@
       <c r="E31" t="n">
         <v>78</v>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1167,6 +1322,11 @@
       <c r="E32" t="n">
         <v>79.5</v>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1190,6 +1350,11 @@
       <c r="E33" t="n">
         <v>81</v>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1213,6 +1378,11 @@
       <c r="E34" t="n">
         <v>82.5</v>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1236,6 +1406,11 @@
       <c r="E35" t="n">
         <v>84</v>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1259,6 +1434,11 @@
       <c r="E36" t="n">
         <v>60</v>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1282,6 +1462,11 @@
       <c r="E37" t="n">
         <v>61.5</v>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1305,6 +1490,11 @@
       <c r="E38" t="n">
         <v>63</v>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1328,6 +1518,11 @@
       <c r="E39" t="n">
         <v>64.5</v>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1351,6 +1546,11 @@
       <c r="E40" t="n">
         <v>66</v>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1374,6 +1574,11 @@
       <c r="E41" t="n">
         <v>67.5</v>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1397,6 +1602,11 @@
       <c r="E42" t="n">
         <v>69</v>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1420,6 +1630,11 @@
       <c r="E43" t="n">
         <v>70.5</v>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1443,6 +1658,11 @@
       <c r="E44" t="n">
         <v>72</v>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1466,6 +1686,11 @@
       <c r="E45" t="n">
         <v>73.5</v>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1489,6 +1714,11 @@
       <c r="E46" t="n">
         <v>75</v>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1512,6 +1742,11 @@
       <c r="E47" t="n">
         <v>76.5</v>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1535,6 +1770,11 @@
       <c r="E48" t="n">
         <v>78</v>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1558,6 +1798,11 @@
       <c r="E49" t="n">
         <v>79.5</v>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1581,6 +1826,11 @@
       <c r="E50" t="n">
         <v>81</v>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1604,6 +1854,11 @@
       <c r="E51" t="n">
         <v>82.5</v>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1627,6 +1882,11 @@
       <c r="E52" t="n">
         <v>84</v>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1650,6 +1910,11 @@
       <c r="E53" t="n">
         <v>60</v>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1673,6 +1938,11 @@
       <c r="E54" t="n">
         <v>61.5</v>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1696,6 +1966,11 @@
       <c r="E55" t="n">
         <v>63</v>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1719,6 +1994,11 @@
       <c r="E56" t="n">
         <v>64.5</v>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1742,6 +2022,11 @@
       <c r="E57" t="n">
         <v>66</v>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1765,6 +2050,11 @@
       <c r="E58" t="n">
         <v>67.5</v>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1788,6 +2078,11 @@
       <c r="E59" t="n">
         <v>69</v>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1811,6 +2106,11 @@
       <c r="E60" t="n">
         <v>70.5</v>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1834,6 +2134,11 @@
       <c r="E61" t="n">
         <v>72</v>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1857,6 +2162,11 @@
       <c r="E62" t="n">
         <v>73.5</v>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1880,6 +2190,11 @@
       <c r="E63" t="n">
         <v>75</v>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1903,6 +2218,11 @@
       <c r="E64" t="n">
         <v>76.5</v>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1926,6 +2246,11 @@
       <c r="E65" t="n">
         <v>78</v>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1949,6 +2274,11 @@
       <c r="E66" t="n">
         <v>79.5</v>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1972,6 +2302,11 @@
       <c r="E67" t="n">
         <v>81</v>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1995,6 +2330,11 @@
       <c r="E68" t="n">
         <v>82.5</v>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2018,6 +2358,11 @@
       <c r="E69" t="n">
         <v>84</v>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2041,6 +2386,11 @@
       <c r="E70" t="n">
         <v>60</v>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2064,6 +2414,11 @@
       <c r="E71" t="n">
         <v>61.5</v>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2087,6 +2442,11 @@
       <c r="E72" t="n">
         <v>63</v>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2110,6 +2470,11 @@
       <c r="E73" t="n">
         <v>64.5</v>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2133,6 +2498,11 @@
       <c r="E74" t="n">
         <v>66</v>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2156,6 +2526,11 @@
       <c r="E75" t="n">
         <v>67.5</v>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2179,6 +2554,11 @@
       <c r="E76" t="n">
         <v>69</v>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2202,6 +2582,11 @@
       <c r="E77" t="n">
         <v>70.5</v>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2225,6 +2610,11 @@
       <c r="E78" t="n">
         <v>72</v>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2248,6 +2638,11 @@
       <c r="E79" t="n">
         <v>73.5</v>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2271,6 +2666,11 @@
       <c r="E80" t="n">
         <v>75</v>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2294,6 +2694,11 @@
       <c r="E81" t="n">
         <v>76.5</v>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2317,6 +2722,11 @@
       <c r="E82" t="n">
         <v>78</v>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2340,6 +2750,11 @@
       <c r="E83" t="n">
         <v>79.5</v>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2363,6 +2778,11 @@
       <c r="E84" t="n">
         <v>81</v>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2386,6 +2806,11 @@
       <c r="E85" t="n">
         <v>82.5</v>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2409,6 +2834,11 @@
       <c r="E86" t="n">
         <v>84</v>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2432,6 +2862,11 @@
       <c r="E87" t="n">
         <v>60</v>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2455,6 +2890,11 @@
       <c r="E88" t="n">
         <v>61.5</v>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2478,6 +2918,11 @@
       <c r="E89" t="n">
         <v>63</v>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2501,6 +2946,11 @@
       <c r="E90" t="n">
         <v>64.5</v>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2524,6 +2974,11 @@
       <c r="E91" t="n">
         <v>66</v>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2547,6 +3002,11 @@
       <c r="E92" t="n">
         <v>67.5</v>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2570,6 +3030,11 @@
       <c r="E93" t="n">
         <v>69</v>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2593,6 +3058,11 @@
       <c r="E94" t="n">
         <v>70.5</v>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2616,6 +3086,11 @@
       <c r="E95" t="n">
         <v>72</v>
       </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2639,6 +3114,11 @@
       <c r="E96" t="n">
         <v>73.5</v>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2662,6 +3142,11 @@
       <c r="E97" t="n">
         <v>75</v>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2685,6 +3170,11 @@
       <c r="E98" t="n">
         <v>76.5</v>
       </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2708,6 +3198,11 @@
       <c r="E99" t="n">
         <v>78</v>
       </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2731,6 +3226,11 @@
       <c r="E100" t="n">
         <v>79.5</v>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2753,6 +3253,11 @@
       </c>
       <c r="E101" t="n">
         <v>81</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Strengthen PivotTable test configuration coverage
</commit_message>
<xml_diff>
--- a/inputs/test_input_100rows.xlsx
+++ b/inputs/test_input_100rows.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,38 +413,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Channel</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Quarter</t>
         </is>
       </c>
     </row>
@@ -487,6 +490,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,6 +533,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -543,6 +576,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -571,6 +619,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -599,6 +662,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -627,6 +705,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -655,6 +748,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -683,6 +791,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -711,6 +834,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -739,6 +877,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -767,6 +920,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -795,6 +963,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -823,6 +1006,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -851,6 +1049,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -879,6 +1092,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -907,6 +1135,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -935,6 +1178,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -963,6 +1221,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -991,6 +1264,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1019,6 +1307,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1047,6 +1350,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1075,6 +1393,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1103,6 +1436,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1131,6 +1479,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1159,6 +1522,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1187,6 +1565,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1215,6 +1608,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1243,6 +1651,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1271,6 +1694,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1299,6 +1737,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1327,6 +1780,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1355,6 +1823,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1383,6 +1866,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1411,6 +1909,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1439,6 +1952,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1467,6 +1995,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1495,6 +2038,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1523,6 +2081,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1551,6 +2124,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1579,6 +2167,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1607,6 +2210,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1635,6 +2253,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1663,6 +2296,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1691,6 +2339,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1719,6 +2382,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1747,6 +2425,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1775,6 +2468,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1803,6 +2511,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1831,6 +2554,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1859,6 +2597,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1887,6 +2640,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1915,6 +2683,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1943,6 +2726,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1971,6 +2769,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1999,6 +2812,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2027,6 +2855,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2055,6 +2898,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2083,6 +2941,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2111,6 +2984,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2139,6 +3027,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2167,6 +3070,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2195,6 +3113,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2223,6 +3156,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2251,6 +3199,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2279,6 +3242,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2307,6 +3285,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2335,6 +3328,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2363,6 +3371,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2391,6 +3414,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2419,6 +3457,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2447,6 +3500,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2475,6 +3543,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2503,6 +3586,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2531,6 +3629,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2559,6 +3672,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2587,6 +3715,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2615,6 +3758,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2643,6 +3801,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2671,6 +3844,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2699,6 +3887,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2727,6 +3930,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2755,6 +3973,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2783,6 +4016,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2811,6 +4059,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2839,6 +4102,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2867,6 +4145,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2895,6 +4188,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2923,6 +4231,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2951,6 +4274,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2979,6 +4317,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3007,6 +4360,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3035,6 +4403,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3063,6 +4446,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3091,6 +4489,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3119,6 +4532,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3147,6 +4575,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3175,6 +4618,21 @@
           <t>Online</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3203,6 +4661,21 @@
           <t>Store</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3231,6 +4704,21 @@
           <t>Partner</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3257,6 +4745,21 @@
       <c r="F101" t="inlineStr">
         <is>
           <t>Online</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Wholesale</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Q1</t>
         </is>
       </c>
     </row>

</xml_diff>